<commit_message>
crm: agregar 5 perfiles nuevos a prospección Instagram (Celular, Mascotas, Viaje, Vivienda, Muebles y Decoración)
</commit_message>
<xml_diff>
--- a/docs/crm-ventas-neggo.xlsx
+++ b/docs/crm-ventas-neggo.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S115"/>
+  <dimension ref="A1:S120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9295,6 +9295,401 @@
         </is>
       </c>
       <c r="S115" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>P-0115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Celulares Medellín 1</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Celular (venta y reparación de celulares, plan retoma)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>@celularesmedellin1 / https://www.instagram.com/celularesmedellin1/</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Medellín (CC Monterrey, Local 089)</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>Bio dice "Más de 10 años de experiencia" y "Plan retoma", 206 mil seguidores, tienda física en CC Monterrey Local 089.</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr">
+        <is>
+          <t>Hola, soy Jhey, fundador de Neggo. Vi la trayectoria de Celulares Medellín: más de 10 años en el CC Monterrey y casi 206 mil seguidores no se construyen de un día para otro. En Neggo conectamos negocios de Medellín con clientes que ya buscan activamente el servicio, como complemento a la demanda que ya generan por su cuenta: pagan solo por resultado real, sin pauta fija ni permanencia. Cada comercio afiliado lleva el Sello de Confianza, que verificamos antes de listarlo. También estamos construyendo Neggo Ads, para pautar en Meta y Google desde el mismo panel — si les interesa quedar en la lista de espera para probarlo primero, avísenme. ¿Hablamos 10 minutos?</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Por enviar</t>
+        </is>
+      </c>
+      <c r="M116" s="3" t="n"/>
+      <c r="N116" s="3" t="n"/>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="R116" s="3" t="inlineStr">
+        <is>
+          <t>Categoría Neggo: Celular. Cuenta grande (206k seguidores, +10 años) — se aplicó tono profesional sección 6.1, mención honesta de Neggo Ads como lista de espera.</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>P-0116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Spot Mascotas</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Mascotas (accesorios y productos)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>@spotmascotas / https://www.instagram.com/spotmascotas/</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Medellín, Antioquia</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>Post reciente explicando por qué nació Spot Mascotas ("un mundo para tu mascota"); bio: accesorios y productos para mascotas, 1.149 seguidores.</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>Hola 👋 vi el post donde cuentan por qué nació Spot Mascotas y se nota el cariño que le ponen a la marca. En Neggo conectamos negocios de Medellín con clientes que ya están buscando accesorios o productos para su mascota, pagando solo por cada lead real, sin pauta ni permanencia. Los comercios afiliados llevan el Sello de Confianza — verificamos cada negocio antes de listarlo, para que el cliente sepa que es real. ¿Te cuento cómo funciona en 5 minutos?</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Por enviar</t>
+        </is>
+      </c>
+      <c r="M117" s="3" t="n"/>
+      <c r="N117" s="3" t="n"/>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="R117" s="3" t="inlineStr">
+        <is>
+          <t>Categoría Neggo: Mascotas. Cuenta regular (1.149 seguidores), tono estándar sección 4.</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>P-0117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Viajes Kaliche</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Viaje (agencia de viajes, RNT 262885)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>@viajeskaliche / https://www.instagram.com/viajeskaliche/</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Medellín / salidas desde Guarne y Niquía</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>Post reciente promocionando plan a Coveñas con salidas desde Guarne y Niquía; bio confirma RNT 262885 (registro nacional de turismo) y 921 seguidores.</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>Hola 👋 vi el plan que armaron a Coveñas saliendo desde Guarne y Niquía, se nota que tienen la logística bien resuelta. En Neggo conectamos agencias como la suya con gente de Medellín que ya está buscando un viaje, pagando solo por lead real entregado, sin pauta ni contrato de permanencia. Como agencia con RNT, califican directo para el Sello de Confianza — verificamos el registro antes de publicarlos, así el viajero sabe que es una agencia real. ¿Charlamos 5 minutos?</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Por enviar</t>
+        </is>
+      </c>
+      <c r="M118" s="3" t="n"/>
+      <c r="N118" s="3" t="n"/>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="R118" s="3" t="inlineStr">
+        <is>
+          <t>Categoría Neggo: Viaje. Cuenta regular (921 seguidores). Ubicación: agencia con salidas Guarne/Niquía (área metro Medellín), verificar con Jhey coherencia geográfica antes de enviar.</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>P-0118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Caza Propia (Juan P. Sánchez)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Vivienda (corretaje inmobiliario)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>@cazapropia.med / https://www.instagram.com/cazapropia.med/</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Medellín, Antioquia</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>Post de lanzamiento explicando el significado de la "Z" en el logo (salir a "cazar" la propiedad en vez de esperar); bio: Agente Inmobiliario certificado, negocio nuevo (publicado 15 jul), 793 seguidores.</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>Hola 👋 me gustó la idea detrás de la "Z" en Caza Propia, se entiende el mensaje de salir a buscar en vez de esperar. Como negocio nuevo, en Neggo podés sumar demanda ya calificada de gente de Medellín buscando comprar o vender vivienda, pagando solo por lead real, sin pauta ni permanencia. Todo comercio afiliado lleva el Sello de Confianza: verificamos tu registro como corredor antes de listarte, para que el cliente sepa que es legítimo. ¿Te cuento cómo funciona?</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Por enviar</t>
+        </is>
+      </c>
+      <c r="M119" s="3" t="n"/>
+      <c r="N119" s="3" t="n"/>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="R119" s="3" t="inlineStr">
+        <is>
+          <t>Categoría Neggo: Vivienda. Cuenta regular (793 seguidores), negocio recién lanzado (jul 2026).</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>P-0119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Decoraciones Imperio</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Muebles y Decoración (fábrica de camas, sofás y persianas)</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>@imperio.decoraciones / https://www.instagram.com/imperio.decoraciones/</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Medellín y Pereira</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>Bio: "Fábrica de Muebles", 707 publicaciones, 8.685 seguidores, presencia en Medellín y Pereira; post activo de oferta de sofá cama con comentarios reales de clientes preguntando precio y medidas.</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t>Hola, soy Jhey, fundador de Neggo. Vi que Decoraciones Imperio ya tiene fábrica propia y presencia en Medellín y Pereira, con casi 8.700 seguidores y actividad constante en el feed, se nota que la producción y las redes ya están resueltas. En Neggo les llevamos demanda adicional ya calificada de gente buscando muebles, como complemento a lo que ya generan ustedes: pagan solo por resultado, sin pauta fija ni permanencia. Cada comercio afiliado lleva el Sello de Confianza, que verificamos antes de listarlo. También estamos construyendo Neggo Ads para pautar en Meta y Google desde el mismo panel — si les interesa quedar en la lista de espera para probarlo primero, les aviso. ¿Hablamos 10 minutos?</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Por enviar</t>
+        </is>
+      </c>
+      <c r="M120" s="3" t="n"/>
+      <c r="N120" s="3" t="n"/>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="R120" s="3" t="inlineStr">
+        <is>
+          <t>Categoría Neggo: Muebles y Decoración. Cuenta grande (8.685 seguidores, 707 publicaciones, fábrica propia) — tono profesional sección 6.1, mención honesta de Neggo Ads como lista de espera.</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>

</xml_diff>